<commit_message>
Expenses: native web-form entry + Exobot area-cost pre-screen + mileage auto-calc + monitoring
Replaces the download/upload Excel flow with a line-item web form (mission-control/expenses.html):
per-line date/category/description/location/amount, mileage auto-computed at the IRS rate
(expense-norms.json). New /api/expense/create runs scripts/expense_screen.py BEFORE routing —
checks each line vs area-normal cost bands (high-cost-metro caps), verifies mileage math,
detects duplicates — and attaches flags to the reviewer's approval task (flagged reports
prioritized + tagged). Adds /api/expense/norms. scripts/expense_analytics.py + monthly
launchd digest report mileage reimbursement per employee and out-of-normal expenses.
Procedure EXOS-ADM-002 updated to rev 1.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -1444,12 +1444,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Exos Expense Report Template (ADM-EXP-01)</t>
+          <t>Mission Control Expenses page; expense-norms.json (area-cost bands + IRS mileage rate)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Aug-10-2026</t>
+          <t>Aug-13-2026</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">

</xml_diff>

<commit_message>
CMMC 2.0: add Cyber Disaster Response & Recovery Plan (PLAN-DR, Draft)
Recovery/continuity half of the CMMC program: scope + RPO(24h)/RTO(4h), roles/invocation,
the nightly asset backup to the attached drive, 3-2-1 posture, step-by-step restore, and
quarterly restore-drill testing. Ties to PLAN-IR/PLAN-RSKRSP/DEF-BSLNCNFG and the
mc-asset-backup engine. Servable in the CMMC 2.0 library.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1457,10 +1457,47 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Cyber Disaster Response &amp; Recovery Plan</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PLAN-DR</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>PLAN-IR (Incident Response), PLAN-RSKRSP (Risk Response), DEF-BSLNCNFG (Baseline Config), SOP-DVCSAN (Sanitization), scripts/mc-asset-backup.py</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Aug-14-2026</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Draft</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DR: capture runtime stack (Brewfile/pip/versions) + New Apple Hardware Rebuild Runbook
Backup now regenerates a system-manifest (Brewfile, pip freeze, versions) each run so a CLEAN
new-Mac install is reproducible. Adds PLAN-DR-HW runbook (CMMC 2.0): verify TM currency ->
Migration Assistant (Path A) or clean install via Brewfile (Path B) -> reconnect Proton/
Cloudflare -> restore+verify mc.db/data -> load the 69 agents -> smoke test. Clarifies the
asset backup is the DATA layer; Time Machine + Migration Assistant is the bare-metal path.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1494,8 +1494,45 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>New Apple Hardware Rebuild Runbook</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PLAN-DR-HW</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>PLAN-DR (Cyber Disaster Response), scripts/mc-asset-backup.py, system-manifest/Brewfile</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Aug-15-2026</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>

</xml_diff>

<commit_message>
Process Library: add EXOS-ADM-003-0 Mission Control Remote Access Onboarding Procedure
Two-layer remote access (Cloudflare Access OTP + MC login), including use from
non-Atomus assets (iPad, home computer) and Atomus-managed devices. Independent
of CMMC/Atomus scope; no CUI in Mission Control.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1531,10 +1531,47 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mission Control Remote Access Onboarding Procedure</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>EXOS-ADM-003-0</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Exos Mission Control (https://mc.exosaero.space); Cloudflare Zero Trust / Access (team soft-hill-c334); Mission Control Admin &gt; Users.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Aug-20-2026</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Approved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Process Library: add EXOS-ADM-004-0 UCR Annual Renewal Procedure
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1568,8 +1568,45 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Unified Carrier Registration (UCR) Annual Renewal</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>EXOS-ADM-004-0</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>USDOT #3020432; www.ucr.gov; MCS-150 (Motor Carrier Identification Report); Unified Carrier Registration program</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Aug-20-2026</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>

</xml_diff>

<commit_message>
Process Library: hold EXOS-ADM-004-0 (UCR Renewal) pending Steve review
Remove from Procedures Master List and mark register/spec 'In Review' per
S. Norsworthy: do not enter into Master List until review complete. Docx and
spec retained; re-add on approval.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1569,44 +1569,6 @@
         </is>
       </c>
       <c r="H29" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Unified Carrier Registration (UCR) Annual Renewal</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>EXOS-ADM-004-0</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>USDOT #3020432; www.ucr.gov; MCS-150 (Motor Carrier Identification Report); Unified Carrier Registration program</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Aug-20-2026</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>

</xml_diff>

<commit_message>
Regenerate procedures on branded letterhead template; commit source specs
The 8 generated procedures rebuilt with the new professional python-docx
template (letterhead header/footer, Calibri, navy section rules, ☐ steps).
Includes their _specs/*.json sources and the refreshed Master List row set.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Aug-13-2026</t>
+          <t>Aug-21-2026</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1466,12 +1466,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cyber Disaster Response &amp; Recovery Plan</t>
+          <t>Mission Control Remote Access Onboarding Procedure</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PLAN-DR</t>
+          <t>EXOS-ADM-003-0</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1481,34 +1481,34 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>PLAN-IR (Incident Response), PLAN-RSKRSP (Risk Response), DEF-BSLNCNFG (Baseline Config), SOP-DVCSAN (Sanitization), scripts/mc-asset-backup.py</t>
+          <t>Exos Mission Control (https://mc.exosaero.space); Cloudflare Zero Trust / Access (team soft-hill-c334); Mission Control Admin &gt; Users.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Aug-14-2026</t>
+          <t>Aug-21-2026</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>New Apple Hardware Rebuild Runbook</t>
+          <t>Unified Carrier Registration (UCR) Annual Renewal</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PLAN-DR-HW</t>
+          <t>EXOS-ADM-004-0</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1518,34 +1518,34 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>PLAN-DR (Cyber Disaster Response), scripts/mc-asset-backup.py, system-manifest/Brewfile</t>
+          <t>USDOT #3020432; www.ucr.gov; MCS-150 (Motor Carrier Identification Report); Unified Carrier Registration program</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Aug-15-2026</t>
+          <t>Aug-21-2026</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>In Review</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mission Control Remote Access Onboarding Procedure</t>
+          <t>ITZ Container Receiving, Offload &amp; Leveling</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EXOS-ADM-003-0</t>
+          <t>EXOS-ITZ-001-0</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1555,12 +1555,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Exos Mission Control (https://mc.exosaero.space); Cloudflare Zero Trust / Access (team soft-hill-c334); Mission Control Admin &gt; Users.</t>
+          <t>DHS CRADA [ref]; Butte (Bert Mooney Airport) ITZ MOA; EXOS-ITZ-002 (Security Monitoring); EXOS-ITZ-003 (Payload Operations); OSHA 29 CFR 1926 Subpart CC (cranes/rigging); OSHA 29 CFR 1910.178 (powered industrial trucks / forklifts).</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aug-20-2026</t>
+          <t>Aug-21-2026</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1570,7 +1570,156 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ITZ Container Security Monitoring System</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>EXOS-ITZ-002-0</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>DHS CRADA [ref]; Butte ITZ MOA; EXOS-ITZ-001; EXOS-ITZ-003; ITZ Technology Control Plan (TCP); ITAR 22 CFR 120-130; EAR 15 CFR 730-774; CMMC 2.0 / NIST SP 800-171 (as applicable); Global Secure Shipping (GSS) training materials.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Aug-21-2026</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ITZ Payload Operations - Inbound Receipt, Outbound Dispatch, and Return</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>EXOS-ITZ-003-0</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>DHS CRADA [ref]; Butte ITZ MOA; ITAR 22 CFR 120-130; EAR 15 CFR 730-774; CBP / Foreign-Trade Zone regulations (19 CFR Part 146); EXOS-ITZ-001; EXOS-ITZ-002. Empowered Official: John Quinn; ITAR reviewer: Denise Shirey.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Aug-21-2026</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>New Apple Hardware Rebuild Runbook</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PLAN-DR-HW</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PLAN-DR (Cyber Disaster Response), scripts/mc-asset-backup.py, system-manifest/Brewfile</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Aug-21-2026</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Cyber Disaster Response &amp; Recovery Plan</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PLAN-DR</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PLAN-IR (Incident Response), PLAN-RSKRSP (Risk Response), DEF-BSLNCNFG (Baseline Config), SOP-DVCSAN (Sanitization), scripts/mc-asset-backup.py</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Aug-21-2026</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Draft</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add EXOS-FIN-001-0 Monthly GAAP Close & Financial Verification procedure
Standard monthly close on QuickBooks (accrual): cutoff, cash/BS reconciliations,
ASC 606 rev rec, flux review, period lock + statement distribution. MC provides
read-only verification on top (not a second ledger). Registered in Process
Library (Finance & Accounting) + assigned monthly close task to Kyle.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1716,8 +1716,45 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Monthly GAAP Close &amp; Financial Verification</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>EXOS-FIN-001-0</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>QuickBooks Online (general ledger / system of record); ASC 606 (revenue recognition); ASC 842 (leases, if applicable); Exos cap table; lender / loan statements; EXOS-ADM-002 Expense Report Submission.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Aug-21-2026</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>

</xml_diff>

<commit_message>
Add EXOS-ADM-005-0 Business Travel and Company Card Procedure
Controlled procedure (house template) covering U.S. + international business
travel and use of the company BILL Divvy Card (Visa Signature Business): card
use, capturing card travel benefits (primary rental CDW, $250k travel accident,
emergency assistance, lost-luggage, concierge, roadside), pay-local-currency,
receipts→QuickBooks, and export/OFAC compliance. Status: Draft (pending owner
approval). Registered in Master List + Process Library. Built via build_procedure.py.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1753,8 +1753,45 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Business Travel and Company Card Procedure</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>EXOS-ADM-005-0</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>BILL Divvy Card Visa Signature Business — Guide to Benefits; EXOS-ADM-002 Expense Report Submission Procedure; current IRS standard mileage rate</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Aug-28-2026</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>

</xml_diff>

<commit_message>
Add EXOS-EXP-001-0 ITAR/EAR-Compliant Supplier Manufacturing Request Procedure (Draft)
US-only, Mission-Control-registered, DD-cleared suppliers only; gates every
controlled-part manufacturing request behind jurisdiction/classification,
supplier eligibility, tech-data marking+minimization, and Empowered Official
release authorization; 5-yr recordkeeping per 22 CFR 122.5. Draft pending EO/
export-counsel review. Built via build_procedure.py onto the house template.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1790,8 +1790,45 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ITAR/EAR-Compliant Supplier Manufacturing Request Procedure</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>EXOS-EXP-001-0</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ITAR, 22 CFR Parts 120-130 (incl. USML 22 CFR 121, DDTC registration 22 CFR 122, recordkeeping 22 CFR 122.5, debarred parties 22 CFR 127.7, U.S. person 22 CFR 120.62); EAR, 15 CFR Parts 730-774 (CCL/ECCN, Denied Persons/Entity List, deemed exports); OFAC SDN and SAM exclusions; Exos Supplier Due Diligence engine and Mission Control supplier DD registry; Exos export-screen / controlled-artifact release path (itar_ear_screen)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Aug-28-2026</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>

</xml_diff>

<commit_message>
Add EXOS-SAF-001-0 Cryogenic LOx Handling Procedure + annual training requirement
Real cryogenic LOx SOP on house template (receipt from Air Products, PPE, storage/
transfer, oxygen-enrichment + cold + pressure hazards, spill/emergency response, annual
re-cert). Registered in Required Reading with recurrence=annual (re-due after 365 days);
replaces the placeholder SAFE-LOX. Draft pending Safety Officer approval.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1827,10 +1827,47 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Cryogenic Oxygen (LOx) Handling Procedure</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>EXOS-SAF-001-0</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Air Products Liquid Oxygen Safety Data Sheet (SDS); Compressed Gas Association CGA P-12 (Safe Handling of Cryogenic Liquids); OSHA 29 CFR 1910 (oxygen / cryogens / PPE); NFPA 55 (Compressed Gases and Cryogenic Fluids Code); Texas Hazard Communication Act (THCA); Exos Emergency Action Plan (SAFE-EAP)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Aug-30-2026</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Draft</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add EXOS-SEC-001-0 AI Tool-Use Policy (tiered: Local / Grok-ZDR / Never)
Bright-line, tiered rule for which AI tool personnel may use per task:
Tier 1 Local (vault, zero egress) for ITAR/EAR/CUI/BD/competitive; Tier 2
Grok enterprise API with ZDR for non-controlled work only; Tier 3 hard
prohibitions. Reflects SpaceX acquisition of xAI (Feb 2026) and no FedRAMP
path. Built via build_procedure.py; on house template, added to Master List
and Process Library. Approved under CEO authority.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1864,8 +1864,45 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>AI Tool-Use Policy (Tiered: Local / Grok-ZDR / Never)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>EXOS-SEC-001-0</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ITAR 22 CFR 120-130 (USML Category IV — launch vehicles &amp; rocket engines, incl. RDRE technical data); EAR 15 CFR 730-774; DFARS 252.204-7012 (CUI safeguarding, NIST SP 800-171); Exos Export-Control Screening (itar_ear_screen); Exos CUI Policies &amp; Procedures (SEC-CUI); xAI/SpaceXAI Zero Data Retention (ZDR) enterprise documentation.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Aug-30-2026</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>

</xml_diff>

<commit_message>
Process Library: add IT-002 Monthly DD-Blocked Senders Outlook Rule Update (Security/CUI)
Controlled procedure (house template, Approved) for each employee to (1) create and
(2) monthly-update an Outlook rule that deletes/junks mail from DD-failed senders,
with safe-use guardrails (never block free-provider domains wholesale). Registered in
the Process Library + Procedures Master List.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1901,8 +1901,45 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Monthly DD-Blocked Senders — Outlook Rule Update</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>IT-002</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Exos DD-Blocked Senders list (issued monthly); CRM Due-Diligence engine; failed-dd-registry</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Sep-02-2026</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>

</xml_diff>

<commit_message>
Add NLX2500 SS Tool Post Calibration procedure (EXOS-MFG-001-0)
New controlled procedure for calibrating the sub-spindle tool setter
(removable arm) on the Mori Seiki NLX2500SY/700 after disc/post
replacement. Creates the 13-manufacturing process-library area.
Also adds initial CNC machine database (data/cnc-machines.json).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1938,8 +1938,45 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>NLX2500 SS Tool Post Calibration</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>EXOS-MFG-001-0</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Mori Seiki / DMG MORI NLX2500SY/700 Operation &amp; Maintenance Manual (sub-spindle tool-eye sensor-position parameters 2097X / 2098X / 2097Z / 2098Z). Machine record: data/cnc-machines.json (NLX2500, SN NL254140428).</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Sep-03-2026</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>

</xml_diff>

<commit_message>
Procedure IT-003: Using Subtasks (Work-Breakdown) in Mission Control (DRAFT)
Authored via build_procedure.py on the house template + Master List +
Process Library. Documents when to use subtasks vs the lightweight
checklist, how to add them (drawer or '@exo subtask:'), roll-up badge,
board/count behavior, and reversible parent tag. DRAFT pending John Quinn
(CEO) approval. Worked example: Part 450 WBS (#2802).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -1975,10 +1975,121 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DCAA-Compliant Timekeeping Policy</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>EXOS-FIN-002-0</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>FAR 31.201; DCAA Contract Audit Manual (DCAM) Ch.5; BambooHR Time Tracking; ERP-exo3 Phase 2</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Sep-05-2026</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>PENDING APPROVAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CUI / ITAR / EAR Document Handling and Storage (SharePoint GCC High)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SEC-CUI-STOR</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>32 CFR Part 2002 (CUI); ITAR 22 CFR 120-130; EAR 15 CFR 730-774; DFARS 252.204-7012; Microsoft 365 GCC High; ERP-exo3 Decision D-002</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Sep-05-2026</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>PENDING APPROVAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Using Subtasks (Work-Breakdown) in Mission Control</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>IT-003</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Mission Control task board; Subtasks feature (shipped 2026-09-10); worked example: BLK3 Part 450 License Application WBS (parent task #2802). Approver: John Quinn (CEO).</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Sep-10-2026</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Draft</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
workspace checkpoint: tracked-file drift across MC data, scripts, capture, drafts & ERP
Checkpoint of 109 tracked changes accumulated across sessions/crons:
- mission-control/data/*.json + pages (decisions, tasks, opportunities, dossiers,
  csl/dd registries, capital_bridge_ledger, erp-rollout, etc.)
- scripts/* automation updates (watchers, capture, dedup, payload engine, IMAP)
- capture/, drafts/, tasks/ content edits and superseded-doc deletions
- erp-foundation (bamboo_sync, dal), config/, HEARTBEAT.md, USER.md
Untracked scratch/generated artifacts (6.3k files) intentionally left unstaged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -2086,10 +2086,47 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>New-Employee Onboarding Procedure (Integrated — HR/BambooHR + Mission Control)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>EXOS-HR-001-0</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>BambooHR (system of record); Exos Mission Control (https://mc.exosaero.space); Cloudflare Zero Trust / One Client (Atomus exosaero team); Payroll: BBSNV (paula.lessnick@bbsnv.com, encrypted Preveil). Automation: scripts/bamboo_newhire_watcher.py (launchd com.exos.bamboo-newhire-watcher, daily). Supersedes legacy 'Exos-US Onboarding Process' (2022).</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Sep-14-2026</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Pending Approval</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Procedure: EXOS-US-MM-001 Materials Management (Procure-to-Pay, Receiving, Inventory, Job Costing)
Documents the end-to-end materials process built this session (QB PO -> Receiving iPad -> inventory/
location/cost -> consume -> per-section job cost -> reconcile to QB). House template, Master List
row, Process Library registered as DRAFT for John's approval; emailed to John.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -2195,8 +2195,43 @@
       <c r="F46" t="b">
         <v>0</v>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Materials Management — Procure-to-Pay, Receiving, Inventory &amp; Job Costing</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>EXOS-US-MM-001</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>QuickBooks (Purchase Orders &amp; Accounts Payable system of record); Mission Control — Receiving / Inventory / Job Cost; BLK3 BOM; Current Inventory Locations map.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Sep-23-2026</t>
+        </is>
+      </c>
+      <c r="F47" t="b">
+        <v>0</v>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>

</xml_diff>

<commit_message>
Procedure: EXOS-US-SEC-VAULT-001 Password Vault (operation/onboarding/admin/backup)
Documents the self-hosted Vaultwarden vault per the standing rule that every new build gets a
procedure + getting-started. House template, Master List, Process Library DRAFT for John; emailed.
Getting-Started guide (Exos_Vault_Getting_Started.pdf) already delivered.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -2230,8 +2230,43 @@
       <c r="F47" t="b">
         <v>0</v>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Password Vault — Operation, Onboarding &amp; Administration</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>EXOS-US-SEC-VAULT-001</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Vaultwarden (self-hosted at https://vault.exosaero.space); official Bitwarden apps; secrets.json key 'vaultwarden_admin_token'; launchd com.exos.vaultwarden-backup; Exos Vault Getting-Started guide.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Sep-23-2026</t>
+        </is>
+      </c>
+      <c r="F48" t="b">
+        <v>0</v>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
         <is>
           <t>DRAFT</t>
         </is>

</xml_diff>

<commit_message>
CM: 23 Atomus CMMC 2.0 docs → Approved (Jon signed 8/13; confirmed 9/26) — register, Master List, Process Library
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -2266,6 +2266,857 @@
         <v>0</v>
       </c>
       <c r="H48" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Audit Events &amp; Logging Definition</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>DEF-AUDITEVNTS</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Baseline Configuration Standard</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>DEF-BSLNCNFG</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Incident Collection Format (DIBNet reporting)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>DEF-ICF</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Security Engineering Principles &amp; System Architecture</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>DEF-SYSENG</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Transactions &amp; Functions by User Role</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>DEF-TRNSFNCS</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Incident Response Plan</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PLAN-IR</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Multi-Factor Authentication Plan</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PLAN-MFA</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Roles &amp; Responsibilities Plan</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>PLAN-ROLESAR</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Risk Response Plan</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PLAN-RSKRSP</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Network Diagram &amp; Assessment Scope</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>CMMC-NETDIAG</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Component Risk Analysis (Automox / Cloudflare / Duo)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>RISK-ANALYSIS</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Change Management SOP</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>SOP-CHNGMGT</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Device &amp; Media Sanitization SOP</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>SOP-DVCSAN</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Information Sensitivity &amp; Data Flow SOP</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SOP-INFSENFLOW</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>System Maintenance SOP</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>SOP-MNTN</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Public Content Posting SOP</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>SOP-PBLCCNTSYS</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Risk Management &amp; Response SOP</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>SOP-RSKMRSPN</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Security Awareness &amp; Training SOP</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SOP-TRNG</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>User Management (Onboarding / Offboarding) SOP</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SOP-USRMGT</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Vulnerability Scanning &amp; Remediation SOP</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SOP-VLNSCNREM</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>IT Systems Review Items &amp; Cadence Plan</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>PLAN-RVWITMS</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Company-Specific Security Values Policy</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>POLICY-CMPNYVAL</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Information Security Policy (master)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>POLICY-ISP</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>CMMC 2.0 Level 2 / NIST SP 800-171r2 / DFARS 252.204-7012; authored by Atomus (v1 Aug-11-2026); master of record in GCC High SharePoint (Exos US-IT-Documents / CMMC Cyber Security)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Aug-13-2026</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>

</xml_diff>

<commit_message>
EXOS-FIN-003-0 Online Invoice Billing & Payment Collection (QuickBooks) — product & payload sales
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -3119,6 +3119,44 @@
       <c r="H71" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Online Invoice Billing &amp; Payment Collection (QuickBooks) - Product &amp; Payload Sales</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>EXOS-FIN-003-0</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>QuickBooks Online + QuickBooks Payments (system of record, card/ACH collection); scripts/qb_invoice.py (prepare / watch); Mission Control Decisions (Approve &amp; send invoice card); mission-control/data/payload-orders.json (payload milestones); product reservation workbooks (e.g. watch workbook); EXOS-FIN-001 Monthly GAAP Close; payload Launch Services Agreement (LSA) milestone schedule.</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Oct-03-2026</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Draft</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CM: SEC-CUI Rev 2 Approved (John Quinn, CEO, 2026-10-08; D-7282008, #3115) — AFRL CUI marking + no-email/DoD SAFE; register, Master List, Process Library; SEC-CUI-STOR email rule aligned
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -3153,10 +3153,46 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>Draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>CUI Policies and Procedures</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>SEC-CUI</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>32 CFR Part 2002 (CUI); DoDI 5200.48; DFARS 252.204-7012 (NIST SP 800-171); AFRL/RJPE CUI marking &amp; DoD SAFE transmission guidance (2026-09-29); SEC-CUI-STOR; Microsoft 365 GCC High</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Oct-08-2026</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Approved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CM: Payload Process Manual Rev4 — approved 2026-10-09 by John Quinn
- Filed Rev4 (PAYLOAD-MAN 1.1 r4) in process-library/03-payload/
- Removed yellow draft highlighting; stamped APPROVED in revision history
- Rev3 (2020-05-28) moved to superseded/
- process-register.json, process-library.html, Procedures_Master_List.xlsx updated
- DOCX + PDF attached to MC task 2957 (doc-keys: payload-process-manual, payload-process-manual__pdf)
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9830" yWindow="3510" windowWidth="25380" windowHeight="15200" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -3193,6 +3193,43 @@
       <c r="H73" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Payload Process Manual v1.1 Rev4</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>PAYLOAD-MAN</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>1.1 r4</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>14 CFR Part 440 (Cross-Waiver of Claims); 14 CFR Part 415/431/450 (payload approval); AC 440.17-1</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Oct-08-2026</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Approved 2026-10-09 by John Quinn, Cofounder &amp; CEO. Added Step #5 Reciprocal Cross-Waiver of Claims (FAA). Supersedes Rev3 (2020-05-28).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SEC-CUI-XFER: add CUI/ITAR/EAR controlled document transfer procedure (DRAFT)
- process-library/08-security-cui/SEC-CUI-XFER_*.docx — new procedure on house template
- process-library/_specs/SEC-CUI-XFER_*.json — generator spec
- Procedures Master List, process-register.json, process-library.html updated
- Decision D-7282033 posted for CEO approval
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9830" yWindow="3510" windowWidth="25380" windowHeight="15200" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -3230,6 +3230,44 @@
       <c r="H74" t="inlineStr">
         <is>
           <t>Approved 2026-10-09 by John Quinn, Cofounder &amp; CEO. Added Step #5 Reciprocal Cross-Waiver of Claims (FAA). Supersedes Rev3 (2020-05-28).</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>CUI / ITAR / EAR Controlled Document Transfer (Internal, Partner, Government)</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SEC-CUI-XFER</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>SEC-CUI-STOR (CUI/ITAR/EAR Document Handling and Storage, SharePoint GCC High); Exos_CUI_Policies_and_Procedures.docx (SEC-CUI Rev 2); EXOS-SEC-001 AI Tool-Use Policy; 22 CFR Parts 120–130 (ITAR) — https://www.ecfr.gov/current/title-22/chapter-I/subchapter-M; 15 CFR Parts 730–774 (EAR) — https://www.ecfr.gov/current/title-15/subtitle-B/chapter-VII/subchapter-C; 22 CFR 122.5 (ITAR recordkeeping) — https://www.ecfr.gov/current/title-22/chapter-I/subchapter-M/part-122/section-122.5; 22 CFR 127.12 (voluntary disclosure) — https://www.ecfr.gov/current/title-22/chapter-I/subchapter-M/part-127/section-127.12; 15 CFR Part 762 (EAR recordkeeping) — https://www.ecfr.gov/current/title-15/subtitle-B/chapter-VII/subchapter-C/part-762; 15 CFR 764.5 (EAR voluntary disclosure) — https://www.ecfr.gov/current/title-15/subtitle-B/chapter-VII/subchapter-C/part-764/section-764.5; 32 CFR Part 2002 (CUI); DFARS 252.204-7012; DoD SAFE — https://safe.apps.mil</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Oct-09-2026</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CM: Payload Process Manual Rev5 — APPROVED 2026-10-11 by John Quinn (D-7282050)
- Filed Rev5 (PAYLOAD-MAN 1.1 r5) in process-library/03-payload/
- Removed yellow draft highlighting; stamped APPROVED 2026-10-11 in revision history
- Rev4 (2026-10-08) moved to superseded/
- process-register.json, cm-register.json, process-library.html, Procedures_Master_List.xlsx updated
- DOCX + PDF attached to MC task 2957 (doc-keys: payload-process-manual-rev5-approved, payload-process-manual-rev5-approved__pdf)
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -3199,7 +3199,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Payload Process Manual v1.1 Rev4</t>
+          <t>Payload Process Manual v1.1 Rev5</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>1.1 r4</t>
+          <t>1.1 r5</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Oct-08-2026</t>
+          <t>Oct-11-2026</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Approved 2026-10-09 by John Quinn, Cofounder &amp; CEO. Added Step #5 Reciprocal Cross-Waiver of Claims (FAA). Supersedes Rev3 (2020-05-28).</t>
+          <t>APPROVED 2026-10-11 by John Quinn, Cofounder &amp; CEO. Rev5: ExoSign default for LPIA; human waiver-on-file confirmation step; in-kind payment path.</t>
         </is>
       </c>
     </row>
@@ -3264,7 +3264,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
           <t>DRAFT</t>

</xml_diff>

<commit_message>
EXOS-FIN-004-0 DRAFT International Contractor Payments & Contractor Expenses (JPY via Wise; BambooHR/Remote backup) for D-7282118 + research memo; CM-on-approval cron 02872e26 registered; build_procedure keeps register format + atomic write
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -3267,6 +3267,44 @@
       <c r="H75" t="inlineStr">
         <is>
           <t>DRAFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>International Contractor Payments &amp; Contractor Expense Reimbursement (incl. JPY)</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>EXOS-FIN-004-0</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>IRS Form W-8BEN (https://www.irs.gov/forms-pubs/about-form-w-8-ben) and W-8BEN-E (https://www.irs.gov/forms-pubs/about-form-w-8-ben-e); IRS withholding on US-source income paid to nonresident aliens (https://www.irs.gov/individuals/international-taxpayers/federal-income-tax-withholding-and-reporting-on-other-kinds-of-us-source-income-paid-to-nonresident-aliens); IRS Pub 515; OFAC Sanctions List Search (https://ofac.treasury.gov/sanctions-list-search-tool); Wise JPY transfer guide (https://wise.com/help/articles/2932156/guide-to-jpy-transfers); Wise-QuickBooks connection (https://wise.com/help/articles/2978059/connect-your-wise-account-with-quickbooks); QuickBooks Online Multicurrency (https://quickbooks.intuit.com/learn-support/en-us/help-article/multicurrency/learn-multicurrency-quickbooks-online/L5krkKQi8_US_en_US); Federal Reserve H.10 (https://www.federalreserve.gov/releases/h10/current); Mission Control Expenses (yen option, scripts/fx_rate.py); EXOS-ADM-002 Expense Report; EXOS-FIN-001 Monthly GAAP Close; CSL denied-party screening (Mission Control); research memo drafts/International_JPY_Payments_Research_2026-10-15.md.</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Oct-15-2026</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Draft</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CM approve EXOS-FIN-004-0 International Contractor Payments (D-7282118)
Procedure approved by John Quinn, Cofounder & CEO via D-7282118.
- Status Draft → Approved; remarks updated
- Rebuilt docx v2, updated Procedures Master List
- Re-registered in cm-register.json (indent-2 canonical form)
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -3293,7 +3293,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Oct-15-2026</t>
+          <t>Oct-16-2026</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3304,7 +3304,7 @@
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EXOS-GRN-008-0 Crane Truck Preventive Maintenance procedure + Freightliner FL112 manuals
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -3301,8 +3301,45 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Crane Truck Preventive Maintenance (1998 Freightliner FL112, Outdoor Storage)</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>EXOS-GRN-008-0</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Freightliner Business Class Trucks Maintenance Manual STI-266 (models FL50-FL112) and Business Class Trucks Driver's Manual (Daimler Trucks North America); crane manufacturer's operator/service manual (pull by crane serial number); engine and transmission manufacturer maintenance manuals; OSHA 29 CFR 1910.180 (crawler, locomotive and truck cranes); OSHA 29 CFR 1926.1412 (crane inspections, used here as the detailed checklist); FMCSA 49 CFR Part 396 (inspection, repair and maintenance); Kobelco Preventative Maintenance Vol. 1, Hydraulic Cylinder (rod protection in storage); EXOS-GRN-001-0 Crane Operations Procedure; EXOS-ADM-004 (UCR registration).</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>

</xml_diff>

<commit_message>
Add EXOS-SALES-002-0 Payload Lead Qualification & Outreach Review + Form F1 (pending John approval, D-7282175)
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -3338,10 +3338,47 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Payload Lead Qualification &amp; Outreach Review</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>EXOS-SALES-002-0</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Form EXOS-SALES-002-F1 Internal Lead Review; BLK3 Payload User's Guide; Exos Past Customer List; EXOS-SALES-001 Sales Agent Commission Procedure; Team Atlas Lead Research Template (S. Mathew, UTD) — student grading tool, not controlled</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Oct-23-2026</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Pending Approval</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Signature gate: wet-ink location must cite File Cabinet/Drawer/Folder (422 otherwise); EXOS-ADM-006-0 site procedure; signing-locations register; exo3 GOVERN registry entry — Jon D-7282192/#4026
</commit_message>
<xml_diff>
--- a/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
+++ b/process-library/01-quality-as9100/Exos_Aerospace_Procedures_Master_List.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34.54296875" bestFit="1" customWidth="1" style="32" min="1" max="1"/>
@@ -3375,10 +3375,47 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>Pending Approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Wet-Ink Signature Document Staging and Location</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>EXOS-ADM-006-0</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Mission Control Decisions (signature gate); mission-control/data/signing-locations.json; Exos DocuSign User Instructions</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Oct-26-2026</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Approved</t>
         </is>
       </c>
     </row>

</xml_diff>